<commit_message>
Apply stash@{0}: WIP state tracking — mark in-pipeline cores as in-use
Adds wip_orders param to DESScheduler, _initialize_wip_state() to pre-mark
cores for orders already at op >= 1300 (already blasted, in pipeline).
Removes WIP orders from blast queue in data_loader so they don't get
rescheduled. Adds wip_in_process_orders to shop_dispatch_parser.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Scheduler Bot Info/Stators Process VSM.xlsx
+++ b/Scheduler Bot Info/Stators Process VSM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SeanFilipow\DD Scheduler Bot\schedulerinfo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SeanFilipow\DD Scheduler Bot\Scheduler Bot Info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71C73E12-10D8-4DFF-8FC6-488A56D47AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13874F9B-0861-4C2D-9C87-103DA311B0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33060" yWindow="2265" windowWidth="29415" windowHeight="15435" activeTab="1" xr2:uid="{5E0B035C-5FA1-4D30-9DFB-4F8251C22B1F}"/>
+    <workbookView xWindow="-705" yWindow="255" windowWidth="28800" windowHeight="15435" activeTab="1" xr2:uid="{5E0B035C-5FA1-4D30-9DFB-4F8251C22B1F}"/>
   </bookViews>
   <sheets>
     <sheet name="Rotors" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
chore: update memory, gitignore debug fixtures, and VSM doc
- memory.md rewritten to reflect MVP 2.0 state (DDSchedulerBot)
- Add debugging-test-uploads/ to .gitignore (contains real client data)
- Minor update to Stators Process VSM.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Scheduler Bot Info/Stators Process VSM.xlsx
+++ b/Scheduler Bot Info/Stators Process VSM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SeanFilipow\DD Scheduler Bot\Scheduler Bot Info\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SeanFilipow\CAMU\ddschedulerbot\Scheduler Bot Info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13874F9B-0861-4C2D-9C87-103DA311B0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183A67B4-5BBE-4431-981E-8901244944EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-705" yWindow="255" windowWidth="28800" windowHeight="15435" activeTab="1" xr2:uid="{5E0B035C-5FA1-4D30-9DFB-4F8251C22B1F}"/>
+    <workbookView xWindow="2475" yWindow="5910" windowWidth="56190" windowHeight="18570" activeTab="1" xr2:uid="{5E0B035C-5FA1-4D30-9DFB-4F8251C22B1F}"/>
   </bookViews>
   <sheets>
     <sheet name="Rotors" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="152">
   <si>
     <t>Type of Rotos</t>
   </si>
@@ -496,6 +496,9 @@
   <si>
     <t>Concurrent with TUBE PREP</t>
   </si>
+  <si>
+    <t>1000 or 1100</t>
+  </si>
 </sst>
 </file>
 
@@ -622,6 +625,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Sheet1"/>
@@ -33960,7 +33964,7 @@
         <v>129</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>77</v>
+        <v>151</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>78</v>

</xml_diff>